<commit_message>
Update FPL data and fix dashboard metrics
</commit_message>
<xml_diff>
--- a/FPL 2025 updated for GW34.xlsx
+++ b/FPL 2025 updated for GW34.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1196f8426b130d45/Desktop/FPL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2357" documentId="11_6E350D49DA2BACEABF531EB1D9C11817159606A2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EC9B07B-F7F0-4D00-AABC-81FE0EE14C09}"/>
+  <xr:revisionPtr revIDLastSave="2360" documentId="11_6E350D49DA2BACEABF531EB1D9C11817159606A2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D8A7F1D-0612-4BCA-A97F-B930520C0DB1}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rules_202625" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="210">
   <si>
     <t>Fantasy Premier League (FPL) Rules</t>
   </si>
@@ -1410,53 +1410,17 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1464,25 +1428,13 @@
     <xf numFmtId="0" fontId="32" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="15" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1519,6 +1471,54 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="15" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -22922,10 +22922,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -25567,7 +25563,7 @@
         <v>250</v>
       </c>
       <c r="G9" s="58">
-        <f>SUM(E9:F9)</f>
+        <f t="shared" ref="G9:G25" si="0">SUM(E9:F9)</f>
         <v>950</v>
       </c>
       <c r="H9" s="58">
@@ -25601,7 +25597,7 @@
         <v>250</v>
       </c>
       <c r="G10" s="58">
-        <f>SUM(E10:F10)</f>
+        <f t="shared" si="0"/>
         <v>950</v>
       </c>
       <c r="H10" s="58">
@@ -25633,7 +25629,7 @@
         <v>250</v>
       </c>
       <c r="G11" s="58">
-        <f>SUM(E11:F11)</f>
+        <f t="shared" si="0"/>
         <v>450</v>
       </c>
       <c r="H11" s="58">
@@ -25667,7 +25663,7 @@
         <v>250</v>
       </c>
       <c r="G12" s="58">
-        <f>SUM(E12:F12)</f>
+        <f t="shared" si="0"/>
         <v>350</v>
       </c>
       <c r="H12" s="58">
@@ -25699,7 +25695,7 @@
         <v>250</v>
       </c>
       <c r="G13" s="58">
-        <f>SUM(E13:F13)</f>
+        <f t="shared" si="0"/>
         <v>950</v>
       </c>
       <c r="H13" s="58">
@@ -25708,7 +25704,7 @@
       </c>
       <c r="I13" s="13">
         <f>COUNTIF('Last Man Paying 2.0'!$E$26:$E$156,Roster!D13)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J13" s="71"/>
     </row>
@@ -25731,7 +25727,7 @@
         <v>250</v>
       </c>
       <c r="G14" s="58">
-        <f>SUM(E14:F14)</f>
+        <f t="shared" si="0"/>
         <v>550</v>
       </c>
       <c r="H14" s="58">
@@ -25740,7 +25736,7 @@
       </c>
       <c r="I14" s="13">
         <f>COUNTIF('Last Man Paying 2.0'!$E$26:$E$156,Roster!D14)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14" s="71"/>
     </row>
@@ -25763,7 +25759,7 @@
         <v>250</v>
       </c>
       <c r="G15" s="58">
-        <f>SUM(E15:F15)</f>
+        <f t="shared" si="0"/>
         <v>750</v>
       </c>
       <c r="H15" s="58">
@@ -25795,7 +25791,7 @@
         <v>250</v>
       </c>
       <c r="G16" s="58">
-        <f>SUM(E16:F16)</f>
+        <f t="shared" si="0"/>
         <v>650</v>
       </c>
       <c r="H16" s="58">
@@ -25829,7 +25825,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="89">
-        <f>SUM(E17:F17)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H17" s="89">
@@ -25863,7 +25859,7 @@
         <v>250</v>
       </c>
       <c r="G18" s="58">
-        <f>SUM(E18:F18)</f>
+        <f t="shared" si="0"/>
         <v>650</v>
       </c>
       <c r="H18" s="58">
@@ -25897,7 +25893,7 @@
         <v>250</v>
       </c>
       <c r="G19" s="58">
-        <f>SUM(E19:F19)</f>
+        <f t="shared" si="0"/>
         <v>950</v>
       </c>
       <c r="H19" s="58">
@@ -25929,7 +25925,7 @@
         <v>250</v>
       </c>
       <c r="G20" s="58">
-        <f>SUM(E20:F20)</f>
+        <f t="shared" si="0"/>
         <v>950</v>
       </c>
       <c r="H20" s="58">
@@ -25961,7 +25957,7 @@
         <v>250</v>
       </c>
       <c r="G21" s="58">
-        <f>SUM(E21:F21)</f>
+        <f t="shared" si="0"/>
         <v>450</v>
       </c>
       <c r="H21" s="58">
@@ -25995,7 +25991,7 @@
         <v>250</v>
       </c>
       <c r="G22" s="58">
-        <f>SUM(E22:F22)</f>
+        <f t="shared" si="0"/>
         <v>1000</v>
       </c>
       <c r="H22" s="58">
@@ -26027,7 +26023,7 @@
         <v>250</v>
       </c>
       <c r="G23" s="58">
-        <f>SUM(E23:F23)</f>
+        <f t="shared" si="0"/>
         <v>650</v>
       </c>
       <c r="H23" s="58">
@@ -26061,7 +26057,7 @@
         <v>250</v>
       </c>
       <c r="G24" s="58">
-        <f>SUM(E24:F24)</f>
+        <f t="shared" si="0"/>
         <v>1050</v>
       </c>
       <c r="H24" s="58">
@@ -26070,7 +26066,7 @@
       </c>
       <c r="I24" s="13">
         <f>COUNTIF('Last Man Paying 2.0'!$E$26:$E$156,Roster!D24)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J24" s="76" t="s">
         <v>51</v>
@@ -26094,7 +26090,7 @@
         <v>250</v>
       </c>
       <c r="G25" s="58">
-        <f>SUM(E25:F25)</f>
+        <f t="shared" si="0"/>
         <v>250</v>
       </c>
       <c r="H25" s="58">
@@ -29237,414 +29233,331 @@
   <sheetFormatPr defaultColWidth="30" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="139"/>
-      <c r="B1" s="141"/>
-      <c r="C1" s="143"/>
+      <c r="A1" s="123"/>
+      <c r="B1" s="125"/>
+      <c r="C1" s="127"/>
       <c r="D1" s="101"/>
       <c r="E1" s="105"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="145"/>
+      <c r="F1" s="146"/>
+      <c r="G1" s="129"/>
     </row>
     <row r="2" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="140"/>
-      <c r="B2" s="142"/>
-      <c r="C2" s="144"/>
+      <c r="A2" s="124"/>
+      <c r="B2" s="126"/>
+      <c r="C2" s="128"/>
       <c r="D2" s="102"/>
       <c r="E2" s="106"/>
-      <c r="F2" s="117"/>
-      <c r="G2" s="146"/>
+      <c r="F2" s="147"/>
+      <c r="G2" s="130"/>
     </row>
     <row r="3" spans="1:7" ht="13.5" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="147"/>
+      <c r="A3" s="131"/>
       <c r="B3" s="103"/>
-      <c r="C3" s="149"/>
-      <c r="D3" s="150"/>
-      <c r="E3" s="150"/>
-      <c r="F3" s="150"/>
-      <c r="G3" s="138"/>
+      <c r="C3" s="133"/>
+      <c r="D3" s="134"/>
+      <c r="E3" s="134"/>
+      <c r="F3" s="134"/>
+      <c r="G3" s="114"/>
     </row>
     <row r="4" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="148"/>
+      <c r="A4" s="132"/>
       <c r="B4" s="107"/>
-      <c r="C4" s="131"/>
-      <c r="D4" s="127"/>
-      <c r="E4" s="127"/>
-      <c r="F4" s="127"/>
-      <c r="G4" s="124"/>
+      <c r="C4" s="119"/>
+      <c r="D4" s="121"/>
+      <c r="E4" s="121"/>
+      <c r="F4" s="121"/>
+      <c r="G4" s="115"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="118"/>
+      <c r="A5" s="116"/>
       <c r="B5" s="103"/>
-      <c r="C5" s="130"/>
-      <c r="D5" s="122"/>
-      <c r="E5" s="122"/>
-      <c r="F5" s="122"/>
-      <c r="G5" s="114"/>
+      <c r="C5" s="118"/>
+      <c r="D5" s="120"/>
+      <c r="E5" s="120"/>
+      <c r="F5" s="120"/>
+      <c r="G5" s="122"/>
     </row>
     <row r="6" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="125"/>
+      <c r="A6" s="117"/>
       <c r="B6" s="107"/>
-      <c r="C6" s="131"/>
-      <c r="D6" s="127"/>
-      <c r="E6" s="127"/>
-      <c r="F6" s="127"/>
-      <c r="G6" s="124"/>
+      <c r="C6" s="119"/>
+      <c r="D6" s="121"/>
+      <c r="E6" s="121"/>
+      <c r="F6" s="121"/>
+      <c r="G6" s="115"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="118"/>
+      <c r="A7" s="116"/>
       <c r="B7" s="103"/>
-      <c r="C7" s="130"/>
-      <c r="D7" s="122"/>
-      <c r="E7" s="122"/>
-      <c r="F7" s="122"/>
-      <c r="G7" s="114"/>
+      <c r="C7" s="118"/>
+      <c r="D7" s="120"/>
+      <c r="E7" s="120"/>
+      <c r="F7" s="120"/>
+      <c r="G7" s="122"/>
     </row>
     <row r="8" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="125"/>
+      <c r="A8" s="117"/>
       <c r="B8" s="107"/>
-      <c r="C8" s="131"/>
-      <c r="D8" s="127"/>
-      <c r="E8" s="127"/>
-      <c r="F8" s="127"/>
-      <c r="G8" s="124"/>
+      <c r="C8" s="119"/>
+      <c r="D8" s="121"/>
+      <c r="E8" s="121"/>
+      <c r="F8" s="121"/>
+      <c r="G8" s="115"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="118"/>
+      <c r="A9" s="116"/>
       <c r="B9" s="103"/>
-      <c r="C9" s="130"/>
-      <c r="D9" s="122"/>
-      <c r="E9" s="122"/>
-      <c r="F9" s="122"/>
-      <c r="G9" s="114"/>
+      <c r="C9" s="118"/>
+      <c r="D9" s="120"/>
+      <c r="E9" s="120"/>
+      <c r="F9" s="120"/>
+      <c r="G9" s="122"/>
     </row>
     <row r="10" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="125"/>
+      <c r="A10" s="117"/>
       <c r="B10" s="107"/>
-      <c r="C10" s="131"/>
-      <c r="D10" s="127"/>
-      <c r="E10" s="127"/>
-      <c r="F10" s="127"/>
-      <c r="G10" s="124"/>
+      <c r="C10" s="119"/>
+      <c r="D10" s="121"/>
+      <c r="E10" s="121"/>
+      <c r="F10" s="121"/>
+      <c r="G10" s="115"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="118"/>
+      <c r="A11" s="116"/>
       <c r="B11" s="103"/>
-      <c r="C11" s="130"/>
-      <c r="D11" s="122"/>
-      <c r="E11" s="122"/>
-      <c r="F11" s="122"/>
-      <c r="G11" s="114"/>
+      <c r="C11" s="118"/>
+      <c r="D11" s="120"/>
+      <c r="E11" s="120"/>
+      <c r="F11" s="120"/>
+      <c r="G11" s="122"/>
     </row>
     <row r="12" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="125"/>
+      <c r="A12" s="117"/>
       <c r="B12" s="107"/>
-      <c r="C12" s="131"/>
-      <c r="D12" s="127"/>
-      <c r="E12" s="127"/>
-      <c r="F12" s="127"/>
-      <c r="G12" s="124"/>
+      <c r="C12" s="119"/>
+      <c r="D12" s="121"/>
+      <c r="E12" s="121"/>
+      <c r="F12" s="121"/>
+      <c r="G12" s="115"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="118"/>
+      <c r="A13" s="116"/>
       <c r="B13" s="103"/>
-      <c r="C13" s="120"/>
-      <c r="D13" s="122"/>
-      <c r="E13" s="122"/>
-      <c r="F13" s="122"/>
-      <c r="G13" s="114"/>
+      <c r="C13" s="135"/>
+      <c r="D13" s="120"/>
+      <c r="E13" s="120"/>
+      <c r="F13" s="120"/>
+      <c r="G13" s="122"/>
     </row>
     <row r="14" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="125"/>
+      <c r="A14" s="117"/>
       <c r="B14" s="107"/>
-      <c r="C14" s="126"/>
-      <c r="D14" s="127"/>
-      <c r="E14" s="127"/>
-      <c r="F14" s="127"/>
-      <c r="G14" s="124"/>
+      <c r="C14" s="136"/>
+      <c r="D14" s="121"/>
+      <c r="E14" s="121"/>
+      <c r="F14" s="121"/>
+      <c r="G14" s="115"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="118"/>
+      <c r="A15" s="116"/>
       <c r="B15" s="103"/>
-      <c r="C15" s="130"/>
-      <c r="D15" s="122"/>
-      <c r="E15" s="122"/>
-      <c r="F15" s="122"/>
-      <c r="G15" s="114"/>
+      <c r="C15" s="118"/>
+      <c r="D15" s="120"/>
+      <c r="E15" s="120"/>
+      <c r="F15" s="120"/>
+      <c r="G15" s="122"/>
     </row>
     <row r="16" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="125"/>
+      <c r="A16" s="117"/>
       <c r="B16" s="107"/>
-      <c r="C16" s="131"/>
-      <c r="D16" s="127"/>
-      <c r="E16" s="127"/>
-      <c r="F16" s="127"/>
-      <c r="G16" s="124"/>
+      <c r="C16" s="119"/>
+      <c r="D16" s="121"/>
+      <c r="E16" s="121"/>
+      <c r="F16" s="121"/>
+      <c r="G16" s="115"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="118"/>
+      <c r="A17" s="116"/>
       <c r="B17" s="103"/>
-      <c r="C17" s="130"/>
-      <c r="D17" s="122"/>
-      <c r="E17" s="122"/>
-      <c r="F17" s="122"/>
-      <c r="G17" s="114"/>
+      <c r="C17" s="118"/>
+      <c r="D17" s="120"/>
+      <c r="E17" s="120"/>
+      <c r="F17" s="120"/>
+      <c r="G17" s="122"/>
     </row>
     <row r="18" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="125"/>
+      <c r="A18" s="117"/>
       <c r="B18" s="107"/>
-      <c r="C18" s="131"/>
-      <c r="D18" s="127"/>
-      <c r="E18" s="127"/>
-      <c r="F18" s="127"/>
-      <c r="G18" s="124"/>
+      <c r="C18" s="119"/>
+      <c r="D18" s="121"/>
+      <c r="E18" s="121"/>
+      <c r="F18" s="121"/>
+      <c r="G18" s="115"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="118"/>
+      <c r="A19" s="116"/>
       <c r="B19" s="103"/>
-      <c r="C19" s="120"/>
-      <c r="D19" s="122"/>
-      <c r="E19" s="122"/>
-      <c r="F19" s="122"/>
-      <c r="G19" s="114"/>
+      <c r="C19" s="135"/>
+      <c r="D19" s="120"/>
+      <c r="E19" s="120"/>
+      <c r="F19" s="120"/>
+      <c r="G19" s="122"/>
     </row>
     <row r="20" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="125"/>
+      <c r="A20" s="117"/>
       <c r="B20" s="107"/>
-      <c r="C20" s="126"/>
-      <c r="D20" s="127"/>
-      <c r="E20" s="127"/>
-      <c r="F20" s="127"/>
-      <c r="G20" s="124"/>
+      <c r="C20" s="136"/>
+      <c r="D20" s="121"/>
+      <c r="E20" s="121"/>
+      <c r="F20" s="121"/>
+      <c r="G20" s="115"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="132"/>
+      <c r="A21" s="137"/>
       <c r="B21" s="108"/>
-      <c r="C21" s="134"/>
-      <c r="D21" s="136"/>
-      <c r="E21" s="136"/>
-      <c r="F21" s="136"/>
-      <c r="G21" s="114"/>
+      <c r="C21" s="139"/>
+      <c r="D21" s="141"/>
+      <c r="E21" s="141"/>
+      <c r="F21" s="141"/>
+      <c r="G21" s="122"/>
     </row>
     <row r="22" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="133"/>
+      <c r="A22" s="138"/>
       <c r="B22" s="104"/>
-      <c r="C22" s="135"/>
-      <c r="D22" s="137"/>
-      <c r="E22" s="137"/>
-      <c r="F22" s="137"/>
-      <c r="G22" s="124"/>
+      <c r="C22" s="140"/>
+      <c r="D22" s="142"/>
+      <c r="E22" s="142"/>
+      <c r="F22" s="142"/>
+      <c r="G22" s="115"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="118"/>
+      <c r="A23" s="116"/>
       <c r="B23" s="103"/>
-      <c r="C23" s="120"/>
-      <c r="D23" s="122"/>
-      <c r="E23" s="122"/>
-      <c r="F23" s="122"/>
-      <c r="G23" s="114"/>
+      <c r="C23" s="135"/>
+      <c r="D23" s="120"/>
+      <c r="E23" s="120"/>
+      <c r="F23" s="120"/>
+      <c r="G23" s="122"/>
     </row>
     <row r="24" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="125"/>
+      <c r="A24" s="117"/>
       <c r="B24" s="107"/>
-      <c r="C24" s="126"/>
-      <c r="D24" s="127"/>
-      <c r="E24" s="127"/>
-      <c r="F24" s="127"/>
-      <c r="G24" s="124"/>
+      <c r="C24" s="136"/>
+      <c r="D24" s="121"/>
+      <c r="E24" s="121"/>
+      <c r="F24" s="121"/>
+      <c r="G24" s="115"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A25" s="118"/>
+      <c r="A25" s="116"/>
       <c r="B25" s="103"/>
-      <c r="C25" s="120"/>
-      <c r="D25" s="122"/>
-      <c r="E25" s="122"/>
-      <c r="F25" s="122"/>
-      <c r="G25" s="114"/>
+      <c r="C25" s="135"/>
+      <c r="D25" s="120"/>
+      <c r="E25" s="120"/>
+      <c r="F25" s="120"/>
+      <c r="G25" s="122"/>
     </row>
     <row r="26" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="125"/>
+      <c r="A26" s="117"/>
       <c r="B26" s="107"/>
-      <c r="C26" s="126"/>
-      <c r="D26" s="127"/>
-      <c r="E26" s="127"/>
-      <c r="F26" s="127"/>
-      <c r="G26" s="124"/>
+      <c r="C26" s="136"/>
+      <c r="D26" s="121"/>
+      <c r="E26" s="121"/>
+      <c r="F26" s="121"/>
+      <c r="G26" s="115"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="118"/>
+      <c r="A27" s="116"/>
       <c r="B27" s="103"/>
-      <c r="C27" s="130"/>
-      <c r="D27" s="122"/>
-      <c r="E27" s="122"/>
-      <c r="F27" s="122"/>
-      <c r="G27" s="114"/>
+      <c r="C27" s="118"/>
+      <c r="D27" s="120"/>
+      <c r="E27" s="120"/>
+      <c r="F27" s="120"/>
+      <c r="G27" s="122"/>
     </row>
     <row r="28" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="125"/>
+      <c r="A28" s="117"/>
       <c r="B28" s="107"/>
-      <c r="C28" s="131"/>
-      <c r="D28" s="127"/>
-      <c r="E28" s="127"/>
-      <c r="F28" s="127"/>
-      <c r="G28" s="124"/>
+      <c r="C28" s="119"/>
+      <c r="D28" s="121"/>
+      <c r="E28" s="121"/>
+      <c r="F28" s="121"/>
+      <c r="G28" s="115"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="118"/>
+      <c r="A29" s="116"/>
       <c r="B29" s="103"/>
-      <c r="C29" s="120"/>
-      <c r="D29" s="122"/>
-      <c r="E29" s="122"/>
-      <c r="F29" s="122"/>
-      <c r="G29" s="128"/>
+      <c r="C29" s="135"/>
+      <c r="D29" s="120"/>
+      <c r="E29" s="120"/>
+      <c r="F29" s="120"/>
+      <c r="G29" s="143"/>
     </row>
     <row r="30" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="125"/>
+      <c r="A30" s="117"/>
       <c r="B30" s="107"/>
-      <c r="C30" s="126"/>
-      <c r="D30" s="127"/>
-      <c r="E30" s="127"/>
-      <c r="F30" s="127"/>
-      <c r="G30" s="129"/>
+      <c r="C30" s="136"/>
+      <c r="D30" s="121"/>
+      <c r="E30" s="121"/>
+      <c r="F30" s="121"/>
+      <c r="G30" s="144"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A31" s="118"/>
+      <c r="A31" s="116"/>
       <c r="B31" s="103"/>
-      <c r="C31" s="120"/>
-      <c r="D31" s="122"/>
-      <c r="E31" s="122"/>
-      <c r="F31" s="122"/>
-      <c r="G31" s="114"/>
+      <c r="C31" s="135"/>
+      <c r="D31" s="120"/>
+      <c r="E31" s="120"/>
+      <c r="F31" s="120"/>
+      <c r="G31" s="122"/>
     </row>
     <row r="32" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="125"/>
+      <c r="A32" s="117"/>
       <c r="B32" s="107"/>
-      <c r="C32" s="126"/>
-      <c r="D32" s="127"/>
-      <c r="E32" s="127"/>
-      <c r="F32" s="127"/>
-      <c r="G32" s="124"/>
+      <c r="C32" s="136"/>
+      <c r="D32" s="121"/>
+      <c r="E32" s="121"/>
+      <c r="F32" s="121"/>
+      <c r="G32" s="115"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A33" s="118"/>
+      <c r="A33" s="116"/>
       <c r="B33" s="103"/>
-      <c r="C33" s="120"/>
-      <c r="D33" s="122"/>
-      <c r="E33" s="122"/>
-      <c r="F33" s="122"/>
-      <c r="G33" s="114"/>
+      <c r="C33" s="135"/>
+      <c r="D33" s="120"/>
+      <c r="E33" s="120"/>
+      <c r="F33" s="120"/>
+      <c r="G33" s="122"/>
     </row>
     <row r="34" spans="1:7" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="125"/>
+      <c r="A34" s="117"/>
       <c r="B34" s="107"/>
-      <c r="C34" s="126"/>
-      <c r="D34" s="127"/>
-      <c r="E34" s="127"/>
-      <c r="F34" s="127"/>
-      <c r="G34" s="124"/>
+      <c r="C34" s="136"/>
+      <c r="D34" s="121"/>
+      <c r="E34" s="121"/>
+      <c r="F34" s="121"/>
+      <c r="G34" s="115"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A35" s="118"/>
+      <c r="A35" s="116"/>
       <c r="B35" s="103"/>
-      <c r="C35" s="120"/>
-      <c r="D35" s="122"/>
-      <c r="E35" s="122"/>
-      <c r="F35" s="122"/>
-      <c r="G35" s="114"/>
+      <c r="C35" s="135"/>
+      <c r="D35" s="120"/>
+      <c r="E35" s="120"/>
+      <c r="F35" s="120"/>
+      <c r="G35" s="122"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A36" s="119"/>
+      <c r="A36" s="148"/>
       <c r="B36" s="107"/>
-      <c r="C36" s="121"/>
-      <c r="D36" s="123"/>
-      <c r="E36" s="123"/>
-      <c r="F36" s="123"/>
-      <c r="G36" s="115"/>
+      <c r="C36" s="149"/>
+      <c r="D36" s="150"/>
+      <c r="E36" s="150"/>
+      <c r="F36" s="150"/>
+      <c r="G36" s="145"/>
     </row>
   </sheetData>
   <mergeCells count="107">
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
     <mergeCell ref="G35:G36"/>
     <mergeCell ref="F1:F2"/>
     <mergeCell ref="A35:A36"/>
@@ -29669,6 +29582,89 @@
     <mergeCell ref="C29:C30"/>
     <mergeCell ref="D29:D30"/>
     <mergeCell ref="E29:E30"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -32481,10 +32477,12 @@
       <c r="C142" s="30">
         <v>1</v>
       </c>
-      <c r="D142" s="29"/>
+      <c r="D142" s="29" t="s">
+        <v>65</v>
+      </c>
       <c r="E142" s="31" t="str">
         <f>IFERROR(VLOOKUP(D142,Roster!$C$8:$D$25,2,),"To be determined")</f>
-        <v>To be determined</v>
+        <v>TAYDO FC</v>
       </c>
       <c r="F142" s="32">
         <v>0</v>
@@ -32499,10 +32497,12 @@
       <c r="C143" s="33">
         <v>2</v>
       </c>
-      <c r="D143" s="29"/>
+      <c r="D143" s="29" t="s">
+        <v>41</v>
+      </c>
       <c r="E143" s="34" t="str">
         <f>IFERROR(VLOOKUP(D143,Roster!$C$8:$D$25,2,),"To be determined")</f>
-        <v>To be determined</v>
+        <v>Hot Slot FC</v>
       </c>
       <c r="F143" s="35">
         <v>0</v>
@@ -32517,10 +32517,12 @@
       <c r="C144" s="36">
         <v>3</v>
       </c>
-      <c r="D144" s="29"/>
+      <c r="D144" s="29" t="s">
+        <v>43</v>
+      </c>
       <c r="E144" s="37" t="str">
         <f>IFERROR(VLOOKUP(D144,Roster!$C$8:$D$25,2,),"To be determined")</f>
-        <v>To be determined</v>
+        <v>Iam_ntombela</v>
       </c>
       <c r="F144" s="38">
         <v>0</v>

</xml_diff>